<commit_message>
fix: keep labeling queue neutral and preserve noise provenance
</commit_message>
<xml_diff>
--- a/templates/labeling_workbook.xlsx
+++ b/templates/labeling_workbook.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="План" sheetId="1" r:id="R465a1648ffb343a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кандидаты" sheetId="2" r:id="R822f812d497747b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Доказательства" sheetId="3" r:id="R6b0dc21b39f14386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="4" r:id="R50f6cd8b0dce495a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шум" sheetId="5" r:id="R24fbf530ac3642f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочник" sheetId="6" r:id="R626a1d69d27443b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="План" sheetId="1" r:id="Rbcda39a27e054ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кандидаты" sheetId="2" r:id="R4093db028a944f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Доказательства" sheetId="3" r:id="Rdbeb2e8a4d204cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="4" r:id="Rd7b011255a2d42b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шум" sheetId="5" r:id="R834c8b3e8e38414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочник" sheetId="6" r:id="R227f454360784791"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -884,7 +884,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Конвейер заполняет идентичность и запрос. Плановый класс задаёт квоту; итоговая метка хранится на листе «Решения».</x:v>
+        <x:v>Конвейер заполняет идентичность и запрос. Класс остаётся пустым до экспертного решения на листе «Решения».</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -900,7 +900,7 @@
         <x:v>candidate_id</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>planned_class</x:v>
+        <x:v>review_pool</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
         <x:v>canonical_name</x:v>
@@ -929,7 +929,7 @@
         <x:v>team-negative-001</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C5" s="25"/>
       <x:c r="D5" s="25"/>
@@ -952,7 +952,7 @@
         <x:v>team-negative-002</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C6" s="25"/>
       <x:c r="D6" s="25"/>
@@ -975,7 +975,7 @@
         <x:v>team-negative-003</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C7" s="25"/>
       <x:c r="D7" s="25"/>
@@ -998,7 +998,7 @@
         <x:v>team-negative-004</x:v>
       </x:c>
       <x:c r="B8" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C8" s="25"/>
       <x:c r="D8" s="25"/>
@@ -1021,7 +1021,7 @@
         <x:v>team-negative-005</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C9" s="25"/>
       <x:c r="D9" s="25"/>
@@ -1044,7 +1044,7 @@
         <x:v>team-negative-006</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C10" s="25"/>
       <x:c r="D10" s="25"/>
@@ -1067,7 +1067,7 @@
         <x:v>team-negative-007</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C11" s="25"/>
       <x:c r="D11" s="25"/>
@@ -1090,7 +1090,7 @@
         <x:v>team-negative-008</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C12" s="25"/>
       <x:c r="D12" s="25"/>
@@ -1113,7 +1113,7 @@
         <x:v>team-negative-009</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C13" s="25"/>
       <x:c r="D13" s="25"/>
@@ -1136,7 +1136,7 @@
         <x:v>team-negative-010</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C14" s="25"/>
       <x:c r="D14" s="25"/>
@@ -1159,7 +1159,7 @@
         <x:v>team-negative-011</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C15" s="25"/>
       <x:c r="D15" s="25"/>
@@ -1182,7 +1182,7 @@
         <x:v>team-negative-012</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C16" s="25"/>
       <x:c r="D16" s="25"/>
@@ -1205,7 +1205,7 @@
         <x:v>team-negative-013</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C17" s="25"/>
       <x:c r="D17" s="25"/>
@@ -1228,7 +1228,7 @@
         <x:v>team-negative-014</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C18" s="25"/>
       <x:c r="D18" s="25"/>
@@ -1251,7 +1251,7 @@
         <x:v>team-negative-015</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C19" s="25"/>
       <x:c r="D19" s="25"/>
@@ -1274,7 +1274,7 @@
         <x:v>team-negative-016</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C20" s="25"/>
       <x:c r="D20" s="25"/>
@@ -1297,7 +1297,7 @@
         <x:v>team-negative-017</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C21" s="25"/>
       <x:c r="D21" s="25"/>
@@ -1320,7 +1320,7 @@
         <x:v>team-negative-018</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C22" s="25"/>
       <x:c r="D22" s="25"/>
@@ -1343,7 +1343,7 @@
         <x:v>team-negative-019</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C23" s="25"/>
       <x:c r="D23" s="25"/>
@@ -1366,7 +1366,7 @@
         <x:v>team-negative-020</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C24" s="25"/>
       <x:c r="D24" s="25"/>
@@ -1389,7 +1389,7 @@
         <x:v>team-negative-021</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C25" s="25"/>
       <x:c r="D25" s="25"/>
@@ -1412,7 +1412,7 @@
         <x:v>team-negative-022</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C26" s="25"/>
       <x:c r="D26" s="25"/>
@@ -1435,7 +1435,7 @@
         <x:v>team-negative-023</x:v>
       </x:c>
       <x:c r="B27" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C27" s="25"/>
       <x:c r="D27" s="25"/>
@@ -1458,7 +1458,7 @@
         <x:v>team-negative-024</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C28" s="25"/>
       <x:c r="D28" s="25"/>
@@ -1481,7 +1481,7 @@
         <x:v>team-negative-025</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C29" s="25"/>
       <x:c r="D29" s="25"/>
@@ -1504,7 +1504,7 @@
         <x:v>team-negative-026</x:v>
       </x:c>
       <x:c r="B30" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C30" s="25"/>
       <x:c r="D30" s="25"/>
@@ -1527,7 +1527,7 @@
         <x:v>team-negative-027</x:v>
       </x:c>
       <x:c r="B31" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C31" s="25"/>
       <x:c r="D31" s="25"/>
@@ -1550,7 +1550,7 @@
         <x:v>team-negative-028</x:v>
       </x:c>
       <x:c r="B32" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C32" s="25"/>
       <x:c r="D32" s="25"/>
@@ -1573,7 +1573,7 @@
         <x:v>team-negative-029</x:v>
       </x:c>
       <x:c r="B33" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C33" s="25"/>
       <x:c r="D33" s="25"/>
@@ -1596,7 +1596,7 @@
         <x:v>team-negative-030</x:v>
       </x:c>
       <x:c r="B34" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C34" s="25"/>
       <x:c r="D34" s="25"/>
@@ -1619,7 +1619,7 @@
         <x:v>team-negative-031</x:v>
       </x:c>
       <x:c r="B35" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C35" s="25"/>
       <x:c r="D35" s="25"/>
@@ -1642,7 +1642,7 @@
         <x:v>team-negative-032</x:v>
       </x:c>
       <x:c r="B36" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C36" s="25"/>
       <x:c r="D36" s="25"/>
@@ -1665,7 +1665,7 @@
         <x:v>team-negative-033</x:v>
       </x:c>
       <x:c r="B37" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C37" s="25"/>
       <x:c r="D37" s="25"/>
@@ -1688,7 +1688,7 @@
         <x:v>team-negative-034</x:v>
       </x:c>
       <x:c r="B38" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C38" s="25"/>
       <x:c r="D38" s="25"/>
@@ -1711,7 +1711,7 @@
         <x:v>team-negative-035</x:v>
       </x:c>
       <x:c r="B39" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C39" s="25"/>
       <x:c r="D39" s="25"/>
@@ -1734,7 +1734,7 @@
         <x:v>team-negative-036</x:v>
       </x:c>
       <x:c r="B40" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C40" s="25"/>
       <x:c r="D40" s="25"/>
@@ -1757,7 +1757,7 @@
         <x:v>team-negative-037</x:v>
       </x:c>
       <x:c r="B41" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C41" s="25"/>
       <x:c r="D41" s="25"/>
@@ -1780,7 +1780,7 @@
         <x:v>team-negative-038</x:v>
       </x:c>
       <x:c r="B42" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C42" s="25"/>
       <x:c r="D42" s="25"/>
@@ -1803,7 +1803,7 @@
         <x:v>team-negative-039</x:v>
       </x:c>
       <x:c r="B43" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C43" s="25"/>
       <x:c r="D43" s="25"/>
@@ -1826,7 +1826,7 @@
         <x:v>team-negative-040</x:v>
       </x:c>
       <x:c r="B44" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C44" s="25"/>
       <x:c r="D44" s="25"/>
@@ -1849,7 +1849,7 @@
         <x:v>team-negative-041</x:v>
       </x:c>
       <x:c r="B45" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C45" s="25"/>
       <x:c r="D45" s="25"/>
@@ -1872,7 +1872,7 @@
         <x:v>team-negative-042</x:v>
       </x:c>
       <x:c r="B46" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C46" s="25"/>
       <x:c r="D46" s="25"/>
@@ -1895,7 +1895,7 @@
         <x:v>team-negative-043</x:v>
       </x:c>
       <x:c r="B47" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C47" s="25"/>
       <x:c r="D47" s="25"/>
@@ -1918,7 +1918,7 @@
         <x:v>team-negative-044</x:v>
       </x:c>
       <x:c r="B48" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C48" s="25"/>
       <x:c r="D48" s="25"/>
@@ -1941,7 +1941,7 @@
         <x:v>team-negative-045</x:v>
       </x:c>
       <x:c r="B49" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C49" s="25"/>
       <x:c r="D49" s="25"/>
@@ -1964,7 +1964,7 @@
         <x:v>team-negative-046</x:v>
       </x:c>
       <x:c r="B50" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C50" s="25"/>
       <x:c r="D50" s="25"/>
@@ -1987,7 +1987,7 @@
         <x:v>team-negative-047</x:v>
       </x:c>
       <x:c r="B51" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C51" s="25"/>
       <x:c r="D51" s="25"/>
@@ -2010,7 +2010,7 @@
         <x:v>team-negative-048</x:v>
       </x:c>
       <x:c r="B52" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C52" s="25"/>
       <x:c r="D52" s="25"/>
@@ -2033,7 +2033,7 @@
         <x:v>team-negative-049</x:v>
       </x:c>
       <x:c r="B53" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C53" s="25"/>
       <x:c r="D53" s="25"/>
@@ -2056,7 +2056,7 @@
         <x:v>team-negative-050</x:v>
       </x:c>
       <x:c r="B54" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C54" s="25"/>
       <x:c r="D54" s="25"/>
@@ -2079,7 +2079,7 @@
         <x:v>team-negative-051</x:v>
       </x:c>
       <x:c r="B55" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C55" s="25"/>
       <x:c r="D55" s="25"/>
@@ -2102,7 +2102,7 @@
         <x:v>team-negative-052</x:v>
       </x:c>
       <x:c r="B56" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C56" s="25"/>
       <x:c r="D56" s="25"/>
@@ -2125,7 +2125,7 @@
         <x:v>team-negative-053</x:v>
       </x:c>
       <x:c r="B57" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C57" s="25"/>
       <x:c r="D57" s="25"/>
@@ -2148,7 +2148,7 @@
         <x:v>team-negative-054</x:v>
       </x:c>
       <x:c r="B58" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C58" s="25"/>
       <x:c r="D58" s="25"/>
@@ -2171,7 +2171,7 @@
         <x:v>team-negative-055</x:v>
       </x:c>
       <x:c r="B59" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C59" s="25"/>
       <x:c r="D59" s="25"/>
@@ -2194,7 +2194,7 @@
         <x:v>team-negative-056</x:v>
       </x:c>
       <x:c r="B60" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C60" s="25"/>
       <x:c r="D60" s="25"/>
@@ -2217,7 +2217,7 @@
         <x:v>team-negative-057</x:v>
       </x:c>
       <x:c r="B61" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C61" s="25"/>
       <x:c r="D61" s="25"/>
@@ -2240,7 +2240,7 @@
         <x:v>team-negative-058</x:v>
       </x:c>
       <x:c r="B62" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C62" s="25"/>
       <x:c r="D62" s="25"/>
@@ -2263,7 +2263,7 @@
         <x:v>team-negative-059</x:v>
       </x:c>
       <x:c r="B63" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C63" s="25"/>
       <x:c r="D63" s="25"/>
@@ -2286,7 +2286,7 @@
         <x:v>team-negative-060</x:v>
       </x:c>
       <x:c r="B64" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C64" s="25"/>
       <x:c r="D64" s="25"/>
@@ -2309,7 +2309,7 @@
         <x:v>team-negative-061</x:v>
       </x:c>
       <x:c r="B65" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C65" s="25"/>
       <x:c r="D65" s="25"/>
@@ -2332,7 +2332,7 @@
         <x:v>team-negative-062</x:v>
       </x:c>
       <x:c r="B66" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C66" s="25"/>
       <x:c r="D66" s="25"/>
@@ -2355,7 +2355,7 @@
         <x:v>team-negative-063</x:v>
       </x:c>
       <x:c r="B67" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C67" s="25"/>
       <x:c r="D67" s="25"/>
@@ -2378,7 +2378,7 @@
         <x:v>team-negative-064</x:v>
       </x:c>
       <x:c r="B68" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C68" s="25"/>
       <x:c r="D68" s="25"/>
@@ -2401,7 +2401,7 @@
         <x:v>team-negative-065</x:v>
       </x:c>
       <x:c r="B69" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C69" s="25"/>
       <x:c r="D69" s="25"/>
@@ -2424,7 +2424,7 @@
         <x:v>team-negative-066</x:v>
       </x:c>
       <x:c r="B70" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C70" s="25"/>
       <x:c r="D70" s="25"/>
@@ -2447,7 +2447,7 @@
         <x:v>team-negative-067</x:v>
       </x:c>
       <x:c r="B71" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C71" s="25"/>
       <x:c r="D71" s="25"/>
@@ -2470,7 +2470,7 @@
         <x:v>team-negative-068</x:v>
       </x:c>
       <x:c r="B72" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C72" s="25"/>
       <x:c r="D72" s="25"/>
@@ -2493,7 +2493,7 @@
         <x:v>team-negative-069</x:v>
       </x:c>
       <x:c r="B73" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C73" s="25"/>
       <x:c r="D73" s="25"/>
@@ -2516,7 +2516,7 @@
         <x:v>team-negative-070</x:v>
       </x:c>
       <x:c r="B74" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C74" s="25"/>
       <x:c r="D74" s="25"/>
@@ -2539,7 +2539,7 @@
         <x:v>team-negative-071</x:v>
       </x:c>
       <x:c r="B75" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C75" s="25"/>
       <x:c r="D75" s="25"/>
@@ -2562,7 +2562,7 @@
         <x:v>team-negative-072</x:v>
       </x:c>
       <x:c r="B76" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C76" s="25"/>
       <x:c r="D76" s="25"/>
@@ -2585,7 +2585,7 @@
         <x:v>team-negative-073</x:v>
       </x:c>
       <x:c r="B77" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C77" s="25"/>
       <x:c r="D77" s="25"/>
@@ -2608,7 +2608,7 @@
         <x:v>team-negative-074</x:v>
       </x:c>
       <x:c r="B78" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C78" s="25"/>
       <x:c r="D78" s="25"/>
@@ -2631,7 +2631,7 @@
         <x:v>team-negative-075</x:v>
       </x:c>
       <x:c r="B79" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C79" s="25"/>
       <x:c r="D79" s="25"/>
@@ -2654,7 +2654,7 @@
         <x:v>team-negative-076</x:v>
       </x:c>
       <x:c r="B80" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C80" s="25"/>
       <x:c r="D80" s="25"/>
@@ -2677,7 +2677,7 @@
         <x:v>team-negative-077</x:v>
       </x:c>
       <x:c r="B81" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C81" s="25"/>
       <x:c r="D81" s="25"/>
@@ -2700,7 +2700,7 @@
         <x:v>team-negative-078</x:v>
       </x:c>
       <x:c r="B82" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C82" s="25"/>
       <x:c r="D82" s="25"/>
@@ -2723,7 +2723,7 @@
         <x:v>team-negative-079</x:v>
       </x:c>
       <x:c r="B83" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C83" s="25"/>
       <x:c r="D83" s="25"/>
@@ -2746,7 +2746,7 @@
         <x:v>team-negative-080</x:v>
       </x:c>
       <x:c r="B84" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C84" s="25"/>
       <x:c r="D84" s="25"/>
@@ -2769,7 +2769,7 @@
         <x:v>team-negative-081</x:v>
       </x:c>
       <x:c r="B85" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C85" s="25"/>
       <x:c r="D85" s="25"/>
@@ -2792,7 +2792,7 @@
         <x:v>team-negative-082</x:v>
       </x:c>
       <x:c r="B86" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C86" s="25"/>
       <x:c r="D86" s="25"/>
@@ -2815,7 +2815,7 @@
         <x:v>team-negative-083</x:v>
       </x:c>
       <x:c r="B87" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C87" s="25"/>
       <x:c r="D87" s="25"/>
@@ -2838,7 +2838,7 @@
         <x:v>team-negative-084</x:v>
       </x:c>
       <x:c r="B88" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C88" s="25"/>
       <x:c r="D88" s="25"/>
@@ -2861,7 +2861,7 @@
         <x:v>team-negative-085</x:v>
       </x:c>
       <x:c r="B89" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C89" s="25"/>
       <x:c r="D89" s="25"/>
@@ -2884,7 +2884,7 @@
         <x:v>team-negative-086</x:v>
       </x:c>
       <x:c r="B90" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C90" s="25"/>
       <x:c r="D90" s="25"/>
@@ -2907,7 +2907,7 @@
         <x:v>team-negative-087</x:v>
       </x:c>
       <x:c r="B91" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C91" s="25"/>
       <x:c r="D91" s="25"/>
@@ -2930,7 +2930,7 @@
         <x:v>team-negative-088</x:v>
       </x:c>
       <x:c r="B92" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C92" s="25"/>
       <x:c r="D92" s="25"/>
@@ -2953,7 +2953,7 @@
         <x:v>team-negative-089</x:v>
       </x:c>
       <x:c r="B93" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C93" s="25"/>
       <x:c r="D93" s="25"/>
@@ -2976,7 +2976,7 @@
         <x:v>team-negative-090</x:v>
       </x:c>
       <x:c r="B94" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C94" s="25"/>
       <x:c r="D94" s="25"/>
@@ -2999,7 +2999,7 @@
         <x:v>team-negative-091</x:v>
       </x:c>
       <x:c r="B95" s="24" t="str">
-        <x:v>mature</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C95" s="25"/>
       <x:c r="D95" s="25"/>
@@ -3022,7 +3022,7 @@
         <x:v>team-negative-092</x:v>
       </x:c>
       <x:c r="B96" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C96" s="25"/>
       <x:c r="D96" s="25"/>
@@ -3045,7 +3045,7 @@
         <x:v>team-negative-093</x:v>
       </x:c>
       <x:c r="B97" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C97" s="25"/>
       <x:c r="D97" s="25"/>
@@ -3068,7 +3068,7 @@
         <x:v>team-negative-094</x:v>
       </x:c>
       <x:c r="B98" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C98" s="25"/>
       <x:c r="D98" s="25"/>
@@ -3091,7 +3091,7 @@
         <x:v>team-negative-095</x:v>
       </x:c>
       <x:c r="B99" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C99" s="25"/>
       <x:c r="D99" s="25"/>
@@ -3114,7 +3114,7 @@
         <x:v>team-negative-096</x:v>
       </x:c>
       <x:c r="B100" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C100" s="25"/>
       <x:c r="D100" s="25"/>
@@ -3137,7 +3137,7 @@
         <x:v>team-negative-097</x:v>
       </x:c>
       <x:c r="B101" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C101" s="25"/>
       <x:c r="D101" s="25"/>
@@ -3160,7 +3160,7 @@
         <x:v>team-negative-098</x:v>
       </x:c>
       <x:c r="B102" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C102" s="25"/>
       <x:c r="D102" s="25"/>
@@ -3183,7 +3183,7 @@
         <x:v>team-negative-099</x:v>
       </x:c>
       <x:c r="B103" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C103" s="25"/>
       <x:c r="D103" s="25"/>
@@ -3206,7 +3206,7 @@
         <x:v>team-negative-100</x:v>
       </x:c>
       <x:c r="B104" s="24" t="str">
-        <x:v>marketing_hype</x:v>
+        <x:v>unclassified</x:v>
       </x:c>
       <x:c r="C104" s="25"/>
       <x:c r="D104" s="25"/>
@@ -3226,8 +3226,8 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B5:B104">
-      <x:formula1>"mature,marketing_hype"</x:formula1>
+    <x:dataValidation type="list" allowBlank="0" showDropDown="1" sqref="B5:B104">
+      <x:formula1>"unclassified"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G5:G104">
       <x:formula1>"Edge,Защита ИИ,Индустриальный ИИ,Инфраструктура ИИ,Роботы,Финтех"</x:formula1>
@@ -3235,7 +3235,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf53b1090ebc54341"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c84b151300140ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12164,7 +12164,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba7c5f816e984c5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09038ba56a074129"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17390,7 +17390,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c5f5747419049fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b0b5fd42f1c4870"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18522,7 +18522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re451570d1f484743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7db11b5889754c23"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>